<commit_message>
Add year view and checkpoint features; enhance README and styling for charts
</commit_message>
<xml_diff>
--- a/tests/fixtures/finances-sample.xlsx
+++ b/tests/fixtures/finances-sample.xlsx
@@ -10,6 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sep 26" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oct 26" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkpoint" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cashflow" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -48,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -582,6 +587,16 @@
         <v>47250</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Bonus</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -850,4 +865,160 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="n">
+        <v>46295</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Savings Accounts</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026 - Monthly Pending</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>300000</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>PPF</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Credit - Ravi</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2027 - Annual Projection</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Savings Accounts</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>450000</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026 - Monthly Pending</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:C20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Sep 26</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Oct 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Opening Balance</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Diwali shopping</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>